<commit_message>
Analyses and figure creation
I have modified the comparative analysis and created figures for the manuscript
</commit_message>
<xml_diff>
--- a/Data/RossSea_Phenology_estimates2025.xlsx
+++ b/Data/RossSea_Phenology_estimates2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/rose_foster-dyer_canterbury_ac_nz/Documents/Github/SAR_RossSea_compare/SAR_RossSea_compare/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="743" documentId="8_{C36C3FC0-118D-426B-A4A0-6E6EFE06D4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FB9C0A5-47E6-4804-BDE6-B5F112F8FEFB}"/>
+  <xr:revisionPtr revIDLastSave="744" documentId="8_{C36C3FC0-118D-426B-A4A0-6E6EFE06D4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C40784D-A320-4B13-AD42-EF5F0C38E411}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D741B97E-D510-4026-838A-5DA85EBB5CBC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{D741B97E-D510-4026-838A-5DA85EBB5CBC}"/>
   </bookViews>
   <sheets>
     <sheet name="full combined" sheetId="9" r:id="rId1"/>
@@ -29640,6 +29640,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updating code and figures
</commit_message>
<xml_diff>
--- a/Data/RossSea_Phenology_estimates2025.xlsx
+++ b/Data/RossSea_Phenology_estimates2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/rose_foster-dyer_canterbury_ac_nz/Documents/Github/SAR_RossSea_compare/SAR_RossSea_compare/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="744" documentId="8_{C36C3FC0-118D-426B-A4A0-6E6EFE06D4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C40784D-A320-4B13-AD42-EF5F0C38E411}"/>
+  <xr:revisionPtr revIDLastSave="746" documentId="8_{C36C3FC0-118D-426B-A4A0-6E6EFE06D4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2842CF00-ADF4-418C-B4AB-77FEC13AA405}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{D741B97E-D510-4026-838A-5DA85EBB5CBC}"/>
+    <workbookView xWindow="28680" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D741B97E-D510-4026-838A-5DA85EBB5CBC}"/>
   </bookViews>
   <sheets>
     <sheet name="full combined" sheetId="9" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'full combined'!$A$1:$AU$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -10944,8 +10945,8 @@
   <dimension ref="A1:AV278"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="40" max="40" width="9.140625" style="6"/>
-    <col min="47" max="47" width="9.140625" style="6"/>
+    <col min="40" max="40" width="13.140625" style="6" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:48" x14ac:dyDescent="0.25">

</xml_diff>